<commit_message>
unifica COLEGIO LA ESPERANZA (IED) DANE 111001098876
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO LA ESPERANZA (IED)-501_Ajustado_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO LA ESPERANZA (IED)-501_Ajustado_CALIFICADO.xlsx
@@ -807,15 +807,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1048,15 +1052,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1297,15 +1305,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -1546,15 +1558,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1719,15 +1735,19 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1968,15 +1988,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2217,15 +2241,19 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -2462,15 +2490,19 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -2711,15 +2743,19 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -2956,15 +2992,19 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3205,15 +3245,19 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -3454,15 +3498,19 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -3663,15 +3711,19 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3908,15 +3960,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4141,15 +4197,19 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4390,15 +4450,19 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4639,15 +4703,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -4888,15 +4956,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -5125,15 +5197,19 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -5374,15 +5450,19 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -5623,15 +5703,19 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -5872,15 +5956,19 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -6121,15 +6209,19 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -6370,15 +6462,19 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -6619,15 +6715,19 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -6868,15 +6968,19 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -7117,15 +7221,19 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -7366,15 +7474,19 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -7615,15 +7727,19 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -7864,15 +7980,19 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8113,15 +8233,19 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -8362,15 +8486,19 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -8611,15 +8739,19 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -8856,15 +8988,19 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9105,15 +9241,19 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9354,15 +9494,19 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -9603,15 +9747,19 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -9852,15 +10000,19 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -10101,15 +10253,19 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -10350,15 +10506,19 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -10595,15 +10755,19 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -10844,15 +11008,19 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -11093,15 +11261,19 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -11342,15 +11514,19 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -11591,15 +11767,19 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -11840,15 +12020,19 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -12089,15 +12273,19 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -12330,15 +12518,19 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -12579,15 +12771,19 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -12828,15 +13024,19 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -13077,15 +13277,19 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -13326,15 +13530,19 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -13571,15 +13779,19 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -13820,15 +14032,19 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -14069,15 +14285,19 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -14318,15 +14538,19 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -14567,15 +14791,19 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -14816,15 +15044,19 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -15065,15 +15297,19 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -15314,15 +15550,19 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED)-SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -15563,15 +15803,19 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -15812,15 +16056,19 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -16061,15 +16309,19 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -16310,15 +16562,19 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr"/>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -16559,15 +16815,19 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -16796,15 +17056,19 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -17045,15 +17309,19 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -17286,15 +17554,19 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -17535,15 +17807,19 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -17776,15 +18052,19 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -18025,15 +18305,19 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -18274,15 +18558,19 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -18523,15 +18811,19 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -18764,15 +19056,19 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -19001,15 +19297,19 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -19230,15 +19530,19 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -19479,15 +19783,19 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -19728,15 +20036,19 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -19977,15 +20289,19 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -20226,15 +20542,19 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>TRATADO</t>
+        </is>
+      </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>111001098878</t>
+          <t>111001098876</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>COLEGIO LA ESPERANZA (IED) - SEDE PRINCIPAL</t>
+          <t>COLEGIO LA ESPERANZA (IED)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">

</xml_diff>